<commit_message>
Random forest con mejor puntaje
</commit_message>
<xml_diff>
--- a/stores/Resultados_random_forest.xlsx
+++ b/stores/Resultados_random_forest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\Academia\Maestría MEcA\Big data y machine learning\Taller 2\ProblemSet2_G10\stores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50601F16-1E6E-4449-A56B-DE1267759AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04763B50-204D-4449-8AA2-7AB7FB2CF630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{6A558E66-D680-4CA7-BD82-ADD54E8BFE60}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
   <si>
     <t>Prueba</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>RF con train_raw sin interacción hacinamiento y n_personas</t>
+  </si>
+  <si>
+    <t>Modelo con mejor puntaje</t>
   </si>
 </sst>
 </file>
@@ -102,7 +105,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -112,6 +115,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -145,16 +154,26 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -172,16 +191,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -515,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC97EA62-D54D-41EF-83DD-100D37B8F67B}">
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="44.59765625" customWidth="1"/>
@@ -523,7 +532,7 @@
     <col min="5" max="5" width="12.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -538,7 +547,7 @@
       </c>
       <c r="K1" s="3"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -569,7 +578,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
@@ -604,7 +613,7 @@
       </c>
       <c r="M3" s="5"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -628,7 +637,7 @@
         <v>10745</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -649,60 +658,74 @@
       </c>
       <c r="M5" s="5"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="9">
         <v>500</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="9">
         <v>4</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
+      <c r="D7" s="9">
+        <v>1</v>
+      </c>
+      <c r="E7" s="9">
         <v>0.93801999999999996</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="9">
         <v>0.871</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="9">
         <v>19421</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="9">
         <v>46747</v>
       </c>
-      <c r="J7" s="1">
+      <c r="I7" s="9"/>
+      <c r="J7" s="10">
         <v>0</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="9">
         <v>32539</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="9">
         <v>3612</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="9">
         <f>L7+K8</f>
         <v>10653</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J8" s="1">
-        <v>1</v>
-      </c>
-      <c r="K8">
+      <c r="N7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="10">
+        <v>1</v>
+      </c>
+      <c r="K8" s="9">
         <v>7041</v>
       </c>
-      <c r="L8">
+      <c r="L8" s="9">
         <v>35968</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="M8" s="9"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A10" s="7" t="s">
         <v>11</v>
       </c>
@@ -742,7 +765,7 @@
         <v>10625</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -763,7 +786,7 @@
       </c>
       <c r="M11" s="5"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A13" s="7" t="s">
         <v>11</v>
       </c>
@@ -803,7 +826,7 @@
         <v>10792</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -824,7 +847,7 @@
       </c>
       <c r="M14" s="5"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A16" s="7" t="s">
         <v>11</v>
       </c>
@@ -1058,32 +1081,31 @@
       <c r="M26" s="5"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28">
         <v>2000</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28">
         <v>8</v>
       </c>
-      <c r="D28" s="9">
-        <v>1</v>
-      </c>
-      <c r="E28" s="9">
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
         <v>0.94562999999999997</v>
       </c>
-      <c r="F28" s="9">
+      <c r="F28">
         <v>0.88490000000000002</v>
       </c>
-      <c r="G28" s="9">
+      <c r="G28">
         <v>18310</v>
       </c>
-      <c r="H28" s="9">
+      <c r="H28">
         <v>47858</v>
       </c>
-      <c r="I28" s="9"/>
-      <c r="J28" s="10">
+      <c r="J28" s="1">
         <v>0</v>
       </c>
       <c r="K28">
@@ -1098,16 +1120,7 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A29" s="9"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="10">
+      <c r="J29" s="1">
         <v>1</v>
       </c>
       <c r="K29">
@@ -1118,16 +1131,16 @@
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31">
         <v>2000</v>
       </c>
-      <c r="C31" s="9">
+      <c r="C31">
         <v>8</v>
       </c>
-      <c r="D31" s="9">
+      <c r="D31">
         <v>1</v>
       </c>
       <c r="E31">
@@ -1142,7 +1155,7 @@
       <c r="H31">
         <v>49213</v>
       </c>
-      <c r="J31" s="10">
+      <c r="J31" s="1">
         <v>0</v>
       </c>
       <c r="K31">
@@ -1157,7 +1170,7 @@
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J32" s="10">
+      <c r="J32" s="1">
         <v>1</v>
       </c>
       <c r="K32">
@@ -1168,7 +1181,7 @@
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B34">
@@ -1192,7 +1205,7 @@
       <c r="H34">
         <v>54530</v>
       </c>
-      <c r="J34" s="10">
+      <c r="J34" s="1">
         <v>0</v>
       </c>
       <c r="K34">
@@ -1207,7 +1220,7 @@
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="J35" s="10">
+      <c r="J35" s="1">
         <v>1</v>
       </c>
       <c r="K35">
@@ -1218,7 +1231,7 @@
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A37" s="8" t="s">
+      <c r="A37" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E37">
@@ -1253,14 +1266,14 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="M4:M80">
-    <cfRule type="top10" dxfId="2" priority="5" bottom="1" rank="1"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="E3:E28">
-    <cfRule type="top10" dxfId="1" priority="2" rank="1"/>
+    <cfRule type="top10" dxfId="2" priority="2" rank="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:F28">
-    <cfRule type="top10" dxfId="0" priority="1" rank="1"/>
+    <cfRule type="top10" dxfId="1" priority="1" rank="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M4:M80">
+    <cfRule type="top10" dxfId="0" priority="5" bottom="1" rank="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>